<commit_message>
docs: cập nhật báo cáo, slide số liệu và kết quả kiểm thử (54/54 TC đạt)
- Chuyển script tạo Excel và báo cáo vào docs/tools
- TC-31 push FCM trên iPhone thật đạt, kèm ảnh màn hình khóa; thêm TC-52..54, BUG-17
- Báo cáo: mục âm báo/chuông, hạn chế iOS, số liệu kiểm thử mới; xuất lại docx và PDF
- Thêm docs/API.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kiem-thu/Ket-qua-kiem-thu.xlsx
+++ b/docs/kiem-thu/Ket-qua-kiem-thu.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test case'!$A$1:$L$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test case'!$A$1:$L$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTA('Test case'!$A$2:$A$99)</f>
+        <f>COUNTA('Test case'!$A$2:$A$105)</f>
         <v/>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$99,"Đạt")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$105,"Đạt")</f>
         <v/>
       </c>
     </row>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$99,"Không đạt")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$105,"Không đạt")</f>
         <v/>
       </c>
     </row>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$99,"Chưa test")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$105,"Chưa test")</f>
         <v/>
       </c>
     </row>
@@ -609,7 +609,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• Kết quả ngày 15/10/2026 lấy từ lần chạy: 53 unit + 57 e2e (Jest) + 23 kịch bản giao diện (Playwright) đều đạt; coverage gộp 94% statements.</t>
+          <t>• Kết quả ngày 15/10/2026 lấy từ lần chạy: 55 unit + 56 e2e (Jest) + 22 kịch bản giao diện (Playwright) đều đạt; coverage gộp 94,5% statements (cập nhật 17/10/2026 sau khi đổi cách người nhà vào xem; 29/10/2026 thêm âm báo, chuông kết thúc, giữ phiên khi mở lại app).</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -832,17 +832,17 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Người nhà nhập mã hợp lệ</t>
+          <t>Người nhà vào xem bằng SĐT + họ tên + tên bệnh nhân</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Nhân viên cấp mã → người nhà nhập mã (chữ thường cũng được)</t>
+          <t>Nhân viên đăng ký người nhà (SĐT + họ tên) → người nhà nhập SĐT, họ tên mình, họ tên bệnh nhân</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Liên kết thành công, thấy bệnh nhân trong danh sách</t>
+          <t>Vào xem được ngay, không mật khẩu; thấy bệnh nhân với tên ẩn bớt</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -852,12 +852,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › TC-03</t>
+          <t>test/family-access.e2e-spec.ts › TC-03; e2e/tests/01-luong-chinh.spec.ts › TC-03</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>201; danh sách có ca, tên hiển thị 'N. V. An'</t>
+          <t>200; danh sách có ca, tên 'N. V. An'; giao diện vào thẳng /theo-doi</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>anh/TC-03.png</t>
+          <t>anh/TC-03.png, anh/TC-03a-nhap-thong-tin.png</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr"/>
@@ -885,37 +885,37 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>FR-06, BR-02</t>
+          <t>FR-07, BR-03</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Người nhà nhập mã hết hạn, đã thu hồi hoặc đã dùng</t>
+          <t>Thông tin không khớp với đăng ký</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Dùng lại mã đã dùng / mã bị thu hồi / mã quá hạn</t>
+          <t>Sai họ tên bệnh nhân / sai họ tên người nhà / SĐT chưa được đăng ký</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Báo lỗi, không tạo liên kết</t>
+          <t>Báo 'chưa khớp với đăng ký của bệnh viện', không vào được</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>API e2e</t>
+          <t>API e2e + UI</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › TC-04 (3 test)</t>
+          <t>test/family-access.e2e-spec.ts › TC-04; e2e/tests/02-loi-va-phien.spec.ts › TC-04</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>400 với thông báo tương ứng cho cả 3 trường hợp</t>
+          <t>401 cho cả 3 trường hợp; giao diện hiện thông báo lỗi</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>anh/TC-04.png, anh/TC-04a-thu-hoi-ma.png</t>
+          <t>anh/TC-04.png</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr"/>
@@ -948,32 +948,32 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Nhập sai mã nhiều lần liên tiếp</t>
+          <t>Nhập sai nhiều lần liên tiếp</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Nhập sai mã 5 lần → lần 6</t>
+          <t>Nhập sai 5 lần với cùng một SĐT → lần 6</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Tạm khóa nhập mã trong một khoảng thời gian</t>
+          <t>Tạm khóa theo SĐT 15 phút</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>API e2e + Unit</t>
+          <t>API e2e + Unit + UI</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › TC-05; attempt-limiter.spec.ts</t>
+          <t>test/family-access.e2e-spec.ts › TC-05; attempt-limiter.spec.ts; e2e/tests/02-loi-va-phien.spec.ts › TC-05</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>5 lần đầu 400, lần 6 trả 429 (khóa 15 phút)</t>
+          <t>401 ×5 rồi 429 'nhập sai quá nhiều lần'</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
@@ -1006,12 +1006,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Người nhà gọi API xem ca chưa liên kết</t>
+          <t>Người nhà xem ca không được đăng ký cho mình</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>GET /my/surgeries/{id}, /surgeries/{id}/history, /surgeries/{id}</t>
+          <t>GET /my/surgeries/{id}, /surgeries/{id}/history, /surgeries/{id} của ca khác</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › TC-06</t>
+          <t>test/family-access.e2e-spec.ts › TC-06</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -1122,32 +1122,32 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Thu hồi liên kết</t>
+          <t>Gỡ quyền theo dõi</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Người nhà bấm 'Ngừng theo dõi' → mở lại chi tiết ca</t>
+          <t>Nhân viên bấm 'Gỡ quyền' (hoặc người nhà 'Ngừng theo dõi') → người nhà mở lại ứng dụng</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Ngừng nhận thông báo và không xem được ca</t>
+          <t>Không xem được nữa; nhập lại thông tin bị từ chối</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>API e2e</t>
+          <t>API e2e + UI</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › TC-08</t>
+          <t>test/family-access.e2e-spec.ts › TC-08; e2e/tests/01-luong-chinh.spec.ts › TC-08</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>204, xem ca trả 404 và không nhận thông báo mới (notifications.e2e BR-05)</t>
+          <t>401 'Phiên theo dõi đã kết thúc'; giao diện về /nguoi-nha, nhập lại báo 'chưa khớp'</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -1291,22 +1291,22 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>FR-01</t>
+          <t>FR-01, FR-07</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Đăng ký tài khoản người nhà</t>
+          <t>Nhân viên đăng ký người nhà cho ca</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Nhập họ tên, SĐT, mật khẩu ≥ 8 ký tự</t>
+          <t>Chi tiết ca → nhập SĐT + họ tên người nhà → Đăng ký</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Tạo tài khoản vai trò người nhà, không trả mật khẩu</t>
+          <t>Người nhà có trong danh sách của ca; SĐT của tài khoản nhân viên bị từ chối</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>test/auth.e2e-spec.ts</t>
+          <t>test/family-access.e2e-spec.ts › staff registers…; e2e/tests/01-luong-chinh.spec.ts › UC-01</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>201, role FAMILY; trùng SĐT trả 409</t>
+          <t>201, danh sách có người nhà; SĐT nhân viên trả 409</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>anh/KQ-02-e2e-test.png</t>
+          <t>anh/UC-01-dang-ky-nguoi-nha.png</t>
         </is>
       </c>
       <c r="K12" s="7" t="inlineStr"/>
@@ -1755,22 +1755,22 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>UC-01</t>
+          <t>Mục 7</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Cấp mã cho ca đã hoàn tất</t>
+          <t>Người nhà vẫn xem trong 24 giờ sau khi ca hoàn tất</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Đi đủ 5 trạng thái → cấp mã</t>
+          <t>Đi đủ 5 trạng thái → người nhà xem chi tiết ca</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Không cho tạo mã mới</t>
+          <t>Vẫn xem được kết quả</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1780,12 +1780,12 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts</t>
+          <t>test/family-access.e2e-spec.ts › BUG-03</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>200 ngay sau khi hoàn tất</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › FR-08; mask-name.spec.ts</t>
+          <t>test/family-access.e2e-spec.ts › FR-08; mask-name.spec.ts</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -1925,33 +1925,37 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>FR-06, FR-07</t>
+          <t>FR-07, NFR-08</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Mở đường dẫn trong QR khi chưa đăng nhập</t>
+          <t>Gõ không dấu, hoa thường, SĐT có khoảng trắng hoặc +84</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Mở /lien-ket?code=... → đăng ký → quay lại</t>
+          <t>Nhập 'tran thi MAI', 'nguyen van an', '+84 901 234 567'</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Sau đăng ký quay về trang liên kết, mã được điền sẵn</t>
+          <t>Vẫn vào xem được</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>UI thủ công</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr"/>
+          <t>API e2e + UI</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>test/family-access.e2e-spec.ts › accepts names…; e2e/tests/02-loi-va-phien.spec.ts › gõ không dấu</t>
+        </is>
+      </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Đúng như mong đợi</t>
+          <t>200; giao diện vào /theo-doi</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -1961,7 +1965,7 @@
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>anh/TC-22.png</t>
+          <t>anh/TC-03b-khong-dau.png</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr"/>
@@ -1984,17 +1988,17 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Không gửi thông báo cho người không còn liên kết</t>
+          <t>Không gửi thông báo cho người không còn quyền</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Người nhà hủy liên kết; người lạ chưa liên kết → đổi trạng thái</t>
+          <t>Nhân viên gỡ quyền một người nhà; người nhà của ca khác → đổi trạng thái</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Cả hai không nhận thông báo</t>
+          <t>Không ai trong hai người nhận thông báo của ca</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2009,7 +2013,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Danh sách thông báo của cả hai rỗng</t>
+          <t>Không có thông báo nào được tạo cho ca</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
@@ -2163,12 +2167,12 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Mở luồng sự kiện của người nhà đã liên kết và người lạ → đổi trạng thái</t>
+          <t>Mở luồng sự kiện của người nhà được đăng ký và của người nhà ca khác → đổi trạng thái</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Chỉ người đã liên kết nhận sự kiện; màn hình đổi ngay</t>
+          <t>Chỉ người được đăng ký nhận sự kiện; màn hình đổi ngay</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2178,12 +2182,12 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>test/events.e2e-spec.ts</t>
+          <t>test/events.e2e-spec.ts; e2e/tests/01-luong-chinh.spec.ts › TC-26</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Người lạ không nhận; qua proxy web nhận ngay, UI cập nhật 113 ms</t>
+          <t>Người ca khác không nhận; màn hình người nhà đổi trong vài trăm ms</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
@@ -2410,7 +2414,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>test/admin.e2e-spec.ts; linking.e2e-spec.ts › FR-11</t>
+          <t>test/admin.e2e-spec.ts; test/family-access.e2e-spec.ts › FR-11</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -2469,17 +2473,25 @@
       <c r="G32" s="6" t="inlineStr"/>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Cần tạo dự án Firebase và điền khóa</t>
+          <t>iPhone (PWA thêm vào màn hình chính) đang tắt màn hình vẫn hiện thông báo 'Bệnh nhân đang được chuyển sang khu vực hồi sức' ngay sau khi đổi trạng thái; FCM trả SENT (dự án Firebase cdtn2-f0527)</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>Chưa test</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="inlineStr"/>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>anh/TC-31a-chuan-bi.png, anh/TC-31b-bat-dau.png, anh/TC-31c-hoi-suc.png, anh/TC-31d-hoan-tat.png</t>
+        </is>
+      </c>
       <c r="K32" s="7" t="inlineStr"/>
-      <c r="L32" s="7" t="inlineStr"/>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2668,22 +2680,22 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Né giới hạn đăng ký bằng token giả</t>
+          <t>Né giới hạn tần suất bằng token giả</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>12 lần đăng ký cùng IP, mỗi lần kèm Bearer ngẫu nhiên</t>
+          <t>Gọi API công khai cùng IP, mỗi lần kèm Bearer ngẫu nhiên</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Bị chặn (429) từ lần thứ 11</t>
+          <t>Token giả bị tính theo IP, không né được giới hạn</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Unit + thủ công (Docker)</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -2693,7 +2705,7 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>201 ×10 rồi 429</t>
+          <t>Đạt (lần kiểm thủ công 15/10 làm trên /auth/register, API này đã bỏ ngày 17/10)</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
@@ -2726,17 +2738,17 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Liên kết với ca đã hoàn tất</t>
+          <t>Không đăng ký thêm người nhà khi ca đã kết thúc</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Cấp mã → hoàn tất ca → nhập mã</t>
+          <t>Hoàn tất ca → nhân viên đăng ký người nhà</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối, báo ca đã kết thúc</t>
+          <t>Bị từ chối</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2746,12 +2758,12 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › BUG-02</t>
+          <t>test/family-access.e2e-spec.ts › UC-01 exception</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>400 'Ca phẫu thuật đã kết thúc'</t>
+          <t>409</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -2784,7 +2796,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Liên kết hết hiệu lực sau khi ca kết thúc</t>
+          <t>Quyền xem hết hiệu lực sau khi ca kết thúc</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2794,7 +2806,7 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Ngay sau vẫn xem được; sau 24 giờ liên kết bị thu hồi</t>
+          <t>Ngay sau vẫn xem được; sau 24 giờ phiên người nhà kết thúc</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2804,12 +2816,12 @@
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › BUG-03</t>
+          <t>test/family-access.e2e-spec.ts › BUG-03</t>
         </is>
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>200 rồi 404, liên kết REVOKED</t>
+          <t>200 rồi 401, liên kết REVOKED</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -2895,33 +2907,37 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>BUG-06</t>
+          <t>FR-02</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Hết phiên khi mở link QR</t>
+          <t>Người nhà không có mật khẩu và không gọi được API nhân viên</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Thu hồi phiên → mở /lien-ket?code=... → bấm Theo dõi → đăng nhập lại</t>
+          <t>Người nhà gọi POST /patients và PUT /auth/password</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Về trang đăng nhập, rồi quay lại đúng trang với mã điền sẵn</t>
+          <t>Bị từ chối do sai vai trò</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>UI thủ công (Docker)</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr"/>
+          <t>API e2e</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>test/auth.e2e-spec.ts › forbids a family member…</t>
+        </is>
+      </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Đúng như mong đợi, liên kết thành công</t>
+          <t>403, 403</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -2931,7 +2947,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>anh/TC-39.png, anh/TC-39a-het-phien.png</t>
+          <t>anh/KQ-02-e2e-test.png</t>
         </is>
       </c>
       <c r="K40" s="7" t="inlineStr"/>
@@ -2949,33 +2965,37 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>BUG-07</t>
+          <t>FR-01</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Đăng nhập với link chuyển hướng sai vai trò</t>
+          <t>Người nhà dùng trang đăng nhập nhân viên</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Mở /dang-nhap?next=/staff, đăng nhập bằng người nhà</t>
+          <t>Nhập SĐT người nhà + mật khẩu bất kỳ ở /dang-nhap</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Về /theo-doi thay vì trang lỗi</t>
+          <t>Bị từ chối; trang có lối sang /nguoi-nha</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>UI thủ công (Docker)</t>
-        </is>
-      </c>
-      <c r="G41" s="6" t="inlineStr"/>
+          <t>API e2e + UI</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>test/auth.e2e-spec.ts › does not let a family member use password login; e2e/tests/02-loi-va-phien.spec.ts › TC-40</t>
+        </is>
+      </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Về /theo-doi</t>
+          <t>401; trang hiện link 'Vào xem bằng số điện thoại'</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -3376,7 +3396,7 @@
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>test/linking.e2e-spec.ts › BUG-15</t>
+          <t>test/family-access.e2e-spec.ts › BUG-15</t>
         </is>
       </c>
       <c r="H48" s="7" t="inlineStr">
@@ -3459,10 +3479,358 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>TC-49</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Có sẵn 3 tài khoản nhân viên và 1 quản trị viên</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Seed → đăng nhập nhanvien1/2/3@benhvien.test, admin@benhvien.test</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Cả 4 tài khoản đăng nhập được, đúng vai trò</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>API e2e</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>test/auth.e2e-spec.ts › seeds 3 staff accounts…</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>200, role STAFF cho cả 3 nhân viên</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>anh/KQ-02-e2e-test.png</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr"/>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>TC-50</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>FR-01</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Bỏ tự đăng ký tài khoản</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>POST /auth/register</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Không còn API tự đăng ký</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>API e2e</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>test/auth.e2e-spec.ts › no longer offers public self-registration</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>anh/KQ-02-e2e-test.png</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>TC-51</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>FR-07</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Một SĐT được đăng ký cho 2 ca</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Nhân viên đăng ký cùng SĐT vào 2 ca → người nhà vào xem 1 lần</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Thấy cả 2 ca</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>API e2e</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>test/family-access.e2e-spec.ts › one phone registered for two surgeries…</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>Danh sách có đủ 2 ca</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>anh/KQ-02-e2e-test.png</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr"/>
+      <c r="L52" s="7" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>TC-52</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Mở lại app khi phiên người nhà còn hạn</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Người nhà vào xem → đóng app → mở lại từ màn hình chính (trang chủ, /nguoi-nha)</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Vào thẳng màn hình theo dõi, không phải nhập lại thông tin</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>UI (Playwright)</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>e2e/tests/07-am-bao-va-phien.spec.ts › TC-52</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển thẳng tới /theo-doi; cookie phiên SameSite=Lax 7 ngày (sửa BUG-17)</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>anh/TC-52-mo-lai-app.png</t>
+        </is>
+      </c>
+      <c r="K53" s="7" t="inlineStr"/>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>TC-53</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>FR-09</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Âm báo khi xong một giai đoạn</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>App người nhà đang mở → nhân viên chuyển 'Đã tiếp nhận' → 'Đang chuẩn bị'</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Kêu một âm báo ngắn và rung nhẹ, không hiện chuông</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>UI (Playwright) + Unit</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>e2e/tests/07-am-bao-va-phien.spec.ts › TC-53; notifications.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>2 nốt âm báo + 1 lần rung; thông báo đẩy mang alert=stage</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>anh/TC-53-am-bao-giai-doan.png</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr"/>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>TC-54</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>FR-09</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Chuông reo khi ca kết thúc</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>App người nhà đang mở → nhân viên chuyển ca tới 'Đã hoàn tất' → bấm 'Tắt chuông'</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Chuông reo và rung lặp lại tới khi người nhà bấm tắt</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>UI (Playwright) + Unit</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>e2e/tests/07-am-bao-va-phien.spec.ts › TC-54</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Hiện bảng 'Ca phẫu thuật đã hoàn tất', chuông lặp mỗi 1,6 giây, dừng hẳn sau khi bấm tắt; push alert=final giữ thông báo trên màn hình (requireInteraction)</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>anh/TC-54-chuong-ket-thuc.png</t>
+        </is>
+      </c>
+      <c r="K55" s="7" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L49"/>
+  <autoFilter ref="A1:L55"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Đạt,Không đạt,Chưa test"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3476,7 +3844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3643,7 +4011,7 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Từ chối liên kết khi ca ở trạng thái cuối</t>
+          <t>Từ chối liên kết khi ca ở trạng thái cuối — Luồng mã/QR đã thay bằng nhân viên đăng ký người nhà (17/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3851,7 +4219,7 @@
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>apiFetch xử lý 401 tập trung, giữ cả query khi chuyển về trang đăng nhập</t>
+          <t>apiFetch xử lý 401 tập trung, giữ cả query khi chuyển về trang đăng nhập — Luồng mã/QR đã thay bằng nhân viên đăng ký người nhà (17/10/2026)</t>
         </is>
       </c>
     </row>
@@ -4378,66 +4746,74 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HC-01</t>
+          <t>BUG-17</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>TC-05, TC-26</t>
+          <t>TC-52</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Bộ đếm nhập sai mã và bus sự kiện SSE lưu trong bộ nhớ: chỉ đúng khi chạy 1 instance API</t>
+          <t>Người nhà mở lại app (PWA trên iPhone) thì phải nhập lại thông tin dù phiên 7 ngày vẫn còn — ảnh anh/BUG-17-mo-lai-app-mat-phien.png</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Chạy 2 instance API sau load balancer</t>
+          <t>Thêm app vào màn hình chính → vào xem → đóng app → mở lại: hiện trang chủ/form nhập thông tin</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Hạn chế đã biết</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr"/>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>ThienBao19</t>
+        </is>
+      </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr"/>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Mở rộng: chuyển sang Redis</t>
+          <t>Trang chủ và /nguoi-nha kiểm tra phiên (GET /auth/me) rồi chuyển thẳng tới trang theo dõi; cookie phiên đổi SameSite=Strict → Lax để vẫn được gửi khi mở app từ màn hình chính hoặc bấm vào thông báo — người dùng phát hiện khi thử trên điện thoại</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HC-02</t>
+          <t>HC-01</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>TC-30</t>
+          <t>TC-05, TC-26</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Chạy dev (không nginx) thì IP trong nhật ký lấy từ X-Forwarded-For do người dùng gửi nên có thể giả</t>
+          <t>Bộ đếm nhập sai mã và bus sự kiện SSE lưu trong bộ nhớ: chỉ đúng khi chạy 1 instance API</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Gọi API qua cổng 3000 kèm X-Forwarded-For tự đặt</t>
+          <t>Chạy 2 instance API sau load balancer</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -4459,29 +4835,29 @@
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Bản triển khai Docker có nginx ghi IP thật</t>
+          <t>Mở rộng: chuyển sang Redis</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>HC-03</t>
+          <t>HC-02</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>TC-14</t>
+          <t>TC-30</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Đăng xuất chỉ xóa cookie trên thiết bị đó; token cũ nếu bị lộ còn dùng được tới hết phiên</t>
+          <t>Chạy dev (không nginx) thì IP trong nhật ký lấy từ X-Forwarded-For do người dùng gửi nên có thể giả</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Sao chép token → đăng xuất → dùng lại token</t>
+          <t>Gọi API qua cổng 3000 kèm X-Forwarded-For tự đặt</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -4503,29 +4879,29 @@
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu để thu hồi mọi phiên</t>
+          <t>Bản triển khai Docker có nginx ghi IP thật</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HC-04</t>
+          <t>HC-03</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>TC-34</t>
+          <t>TC-14</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Giới hạn đăng nhập theo tài khoản: người khác cố tình đăng nhập sai có thể làm tài khoản bị chặn 1 phút</t>
+          <t>Đăng xuất chỉ xóa cookie trên thiết bị đó; token cũ nếu bị lộ còn dùng được tới hết phiên</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Đăng nhập sai 10 lần vào tài khoản của người khác</t>
+          <t>Sao chép token → đăng xuất → dùng lại token</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -4547,34 +4923,34 @@
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Đánh đổi để chống dò mật khẩu</t>
+          <t>Đổi mật khẩu để thu hồi mọi phiên</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HC-05</t>
+          <t>HC-04</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>TC-31</t>
+          <t>TC-34</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Chưa thử push FCM trên điện thoại thật vì chưa có dự án Firebase</t>
+          <t>Giới hạn đăng nhập theo tài khoản: người khác cố tình đăng nhập sai có thể làm tài khoản bị chặn 1 phút</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Đăng nhập sai 10 lần vào tài khoản của người khác</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -4591,29 +4967,29 @@
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Thông báo vẫn hiện trong ứng dụng qua SSE</t>
+          <t>Đánh đổi để chống dò mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>HC-06</t>
+          <t>HC-05</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>KQ-01</t>
+          <t>TC-31, TC-54</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Jest báo 'worker failed to exit gracefully' khi chạy unit test song song trên Windows (do nạp Prisma/throttler), không ảnh hưởng kết quả</t>
+          <t>iPhone không cho web rung máy; khi app đang đóng hệ điều hành chỉ phát âm thông báo mặc định một lần, chuông lặp chỉ có khi app đang mở</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>pnpm --filter @pt/api test</t>
+          <t>Tắt app trên iPhone → nhân viên chuyển ca sang 'Đã hoàn tất'</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -4629,13 +5005,101 @@
       <c r="G23" s="6" t="inlineStr"/>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="6" t="inlineStr">
         <is>
+          <t>Giới hạn của web push trên iOS; Android vẫn rung dài và giữ thông báo tới khi người dùng tắt</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>HC-06</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>KQ-01</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Jest báo 'worker failed to exit gracefully' khi chạy unit test song song trên Windows (do nạp Prisma/throttler), không ảnh hưởng kết quả</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>pnpm --filter @pt/api test</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Hạn chế đã biết</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr">
+        <is>
           <t>Chạy tuần tự (--runInBand) và --detectOpenHandles không thấy rò rỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>HC-07</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>TC-03, TC-05</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Người nhà vào xem không cần mật khẩu: ai biết đúng SĐT, họ tên người nhà và họ tên bệnh nhân đã được đăng ký thì xem được</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Nhập đúng 3 thông tin của một người nhà đã được đăng ký</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Hạn chế đã biết</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Theo yêu cầu (không mật khẩu, không xác nhận). Giảm thiểu: chỉ người nhân viên đăng ký mới vào được, khóa 5 lần sai/15 phút theo SĐT, phiên hết khi ca kết thúc, nhật ký FAMILY_ACCESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: thêm BUG-18, TC-55 và cập nhật số liệu kiểm thử (55/55 TC đạt)
</commit_message>
<xml_diff>
--- a/docs/kiem-thu/Ket-qua-kiem-thu.xlsx
+++ b/docs/kiem-thu/Ket-qua-kiem-thu.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug log" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test case'!$A$1:$L$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test case'!$A$1:$L$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -498,7 +498,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTA('Test case'!$A$2:$A$105)</f>
+        <f>COUNTA('Test case'!$A$2:$A$106)</f>
         <v/>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$105,"Đạt")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$106,"Đạt")</f>
         <v/>
       </c>
     </row>
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$105,"Không đạt")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$106,"Không đạt")</f>
         <v/>
       </c>
     </row>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <f>COUNTIF('Test case'!$I$2:$I$105,"Chưa test")</f>
+        <f>COUNTIF('Test case'!$I$2:$I$106,"Chưa test")</f>
         <v/>
       </c>
     </row>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3827,10 +3827,68 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>TC-55</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>FR-09</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Đổi người nhà trên cùng điện thoại vẫn nhận push</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Điện thoại đã bật thông báo cho người nhà A → người nhà B vào xem trên cùng máy → nhân viên đổi trạng thái ca của B, tắt màn hình</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Thông báo của B hiện trên màn hình khóa</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>API e2e + Thủ công</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>test/notifications.e2e-spec.ts › TC-55</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>Mở app thì token chuyển sang B; 4 thông báo ca thử 31/10 đều SENT tới iPhone</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>anh/KQ-02-e2e-test.png</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr"/>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L55"/>
+  <autoFilter ref="A1:L56"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Đạt,Không đạt,Chưa test"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3844,7 +3902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4798,66 +4856,74 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HC-01</t>
+          <t>BUG-18</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>TC-05, TC-26</t>
+          <t>TC-55</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Bộ đếm nhập sai mã và bus sự kiện SSE lưu trong bộ nhớ: chỉ đúng khi chạy 1 instance API</t>
+          <t>Người nhà thứ hai vào xem trên điện thoại đã bật thông báo thì không nhận push (bị ghi SKIPPED)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Chạy 2 instance API sau load balancer</t>
+          <t>Bật thông báo khi vào bằng người nhà A → vào bằng người nhà B trên cùng máy → đổi trạng thái ca của B</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Hạn chế đã biết</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr"/>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>ThienBao19</t>
+        </is>
+      </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr"/>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Mở rộng: chuyển sang Redis</t>
+          <t>Token thiết bị vẫn gắn với A vì nút Cài đặt hiện 'đang bật' nên không đăng ký lại; nay mỗi lần mở app tự đăng ký lại token cho người đang vào xem — người dùng phát hiện khi thử trên điện thoại</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>HC-02</t>
+          <t>HC-01</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>TC-30</t>
+          <t>TC-05, TC-26</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Chạy dev (không nginx) thì IP trong nhật ký lấy từ X-Forwarded-For do người dùng gửi nên có thể giả</t>
+          <t>Bộ đếm nhập sai mã và bus sự kiện SSE lưu trong bộ nhớ: chỉ đúng khi chạy 1 instance API</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Gọi API qua cổng 3000 kèm X-Forwarded-For tự đặt</t>
+          <t>Chạy 2 instance API sau load balancer</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -4879,29 +4945,29 @@
       <c r="I20" s="6" t="inlineStr"/>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Bản triển khai Docker có nginx ghi IP thật</t>
+          <t>Mở rộng: chuyển sang Redis</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HC-03</t>
+          <t>HC-02</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>TC-14</t>
+          <t>TC-30</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Đăng xuất chỉ xóa cookie trên thiết bị đó; token cũ nếu bị lộ còn dùng được tới hết phiên</t>
+          <t>Chạy dev (không nginx) thì IP trong nhật ký lấy từ X-Forwarded-For do người dùng gửi nên có thể giả</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Sao chép token → đăng xuất → dùng lại token</t>
+          <t>Gọi API qua cổng 3000 kèm X-Forwarded-For tự đặt</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -4923,29 +4989,29 @@
       <c r="I21" s="6" t="inlineStr"/>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu để thu hồi mọi phiên</t>
+          <t>Bản triển khai Docker có nginx ghi IP thật</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HC-04</t>
+          <t>HC-03</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>TC-34</t>
+          <t>TC-14</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Giới hạn đăng nhập theo tài khoản: người khác cố tình đăng nhập sai có thể làm tài khoản bị chặn 1 phút</t>
+          <t>Đăng xuất chỉ xóa cookie trên thiết bị đó; token cũ nếu bị lộ còn dùng được tới hết phiên</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Đăng nhập sai 10 lần vào tài khoản của người khác</t>
+          <t>Sao chép token → đăng xuất → dùng lại token</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
@@ -4967,29 +5033,29 @@
       <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Đánh đổi để chống dò mật khẩu</t>
+          <t>Đổi mật khẩu để thu hồi mọi phiên</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>HC-05</t>
+          <t>HC-04</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>TC-31, TC-54</t>
+          <t>TC-34</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>iPhone không cho web rung máy; khi app đang đóng hệ điều hành chỉ phát âm thông báo mặc định một lần, chuông lặp chỉ có khi app đang mở</t>
+          <t>Giới hạn đăng nhập theo tài khoản: người khác cố tình đăng nhập sai có thể làm tài khoản bị chặn 1 phút</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Tắt app trên iPhone → nhân viên chuyển ca sang 'Đã hoàn tất'</t>
+          <t>Đăng nhập sai 10 lần vào tài khoản của người khác</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -5011,29 +5077,29 @@
       <c r="I23" s="6" t="inlineStr"/>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Giới hạn của web push trên iOS; Android vẫn rung dài và giữ thông báo tới khi người dùng tắt</t>
+          <t>Đánh đổi để chống dò mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>HC-06</t>
+          <t>HC-05</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>KQ-01</t>
+          <t>TC-31, TC-54</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Jest báo 'worker failed to exit gracefully' khi chạy unit test song song trên Windows (do nạp Prisma/throttler), không ảnh hưởng kết quả</t>
+          <t>iPhone không cho web rung máy; khi app đang đóng hệ điều hành chỉ phát âm thông báo mặc định một lần, chuông lặp chỉ có khi app đang mở</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>pnpm --filter @pt/api test</t>
+          <t>Tắt app trên iPhone → nhân viên chuyển ca sang 'Đã hoàn tất'</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -5049,40 +5115,40 @@
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Chạy tuần tự (--runInBand) và --detectOpenHandles không thấy rò rỉ</t>
+          <t>Giới hạn của web push trên iOS; Android vẫn rung dài và giữ thông báo tới khi người dùng tắt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>HC-07</t>
+          <t>HC-06</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>TC-03, TC-05</t>
+          <t>KQ-01</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Người nhà vào xem không cần mật khẩu: ai biết đúng SĐT, họ tên người nhà và họ tên bệnh nhân đã được đăng ký thì xem được</t>
+          <t>Jest báo 'worker failed to exit gracefully' khi chạy unit test song song trên Windows (do nạp Prisma/throttler), không ảnh hưởng kết quả</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Nhập đúng 3 thông tin của một người nhà đã được đăng ký</t>
+          <t>pnpm --filter @pt/api test</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -5093,11 +5159,55 @@
       <c r="G25" s="6" t="inlineStr"/>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>17/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Chạy tuần tự (--runInBand) và --detectOpenHandles không thấy rò rỉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>HC-07</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>TC-03, TC-05</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Người nhà vào xem không cần mật khẩu: ai biết đúng SĐT, họ tên người nhà và họ tên bệnh nhân đã được đăng ký thì xem được</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Nhập đúng 3 thông tin của một người nhà đã được đăng ký</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Hạn chế đã biết</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>Theo yêu cầu (không mật khẩu, không xác nhận). Giảm thiểu: chỉ người nhân viên đăng ký mới vào được, khóa 5 lần sai/15 phút theo SĐT, phiên hết khi ca kết thúc, nhật ký FAMILY_ACCESS</t>
         </is>

</xml_diff>